<commit_message>
Task 2: comprehensive market-wise EDA workbook (docs/EDA.xlsx)
- eda.py: per-market tables (channel share, category split, weekday/monthly
  seasonality, promo/holiday/weekend uplift, top brands, intermittency-by-channel)
  + cross-market tables (summary, channel mix %, uplift, weather corr)
- scripts/make_eda_workbook.py -> docs/EDA.xlsx (Overview + 4 market sheets +
  4 cross-market sheets); wired into 'make eda'
- tests for market-wise tables; Task2_Summary references EDA.xlsx
</commit_message>
<xml_diff>
--- a/docs/Task2_Summary.xlsx
+++ b/docs/Task2_Summary.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>7 figures in docs/eda/, findings in docs/eda_findings.md, and this workbook.</t>
+          <t>Market-wise docs/EDA.xlsx (per-market + cross-market sheets), 7 figures in docs/eda/, findings in docs/eda_findings.md, and this workbook.</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1276,7 +1276,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Figures (docs/eda/) + findings doc</t>
+          <t>Market-wise EDA workbook (docs/EDA.xlsx)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1288,7 +1288,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Fixed 2 generator bugs found via EDA</t>
+          <t>Figures (docs/eda/) + findings doc</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1300,10 +1300,22 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Fixed 2 generator bugs found via EDA</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
           <t>Task2_Summary.xlsx (this file)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>

</xml_diff>